<commit_message>
Refinements made to age groups and monthly cost calculations
</commit_message>
<xml_diff>
--- a/ILSA_running_budget.xlsx
+++ b/ILSA_running_budget.xlsx
@@ -958,7 +958,7 @@
         <v>183879</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>1000</v>
+        <v>1099</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>21</v>
@@ -1565,12 +1565,14 @@
       <c r="B9" s="31" t="n">
         <v>370</v>
       </c>
-      <c r="C9" s="32" t="n"/>
+      <c r="C9" s="32" t="n">
+        <v>273</v>
+      </c>
       <c r="D9" s="21" t="n">
         <v>900</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>783.38</v>
+        <v>634.8099999999999</v>
       </c>
       <c r="F9" s="21">
         <f>IF(E9="","",D9-E9)</f>
@@ -1590,12 +1592,14 @@
       <c r="B10" s="35" t="n">
         <v>425</v>
       </c>
-      <c r="C10" s="36" t="n"/>
+      <c r="C10" s="36" t="n">
+        <v>324</v>
+      </c>
       <c r="D10" s="23" t="n">
         <v>1000</v>
       </c>
       <c r="E10" s="37" t="n">
-        <v>904.09</v>
+        <v>783.38</v>
       </c>
       <c r="F10" s="23">
         <f>IF(E10="","",D10-E10)</f>
@@ -1615,12 +1619,14 @@
       <c r="B11" s="31" t="n">
         <v>490</v>
       </c>
-      <c r="C11" s="32" t="n"/>
+      <c r="C11" s="32" t="n">
+        <v>379</v>
+      </c>
       <c r="D11" s="21" t="n">
         <v>1200</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>1010.92</v>
+        <v>904.09</v>
       </c>
       <c r="F11" s="21">
         <f>IF(E11="","",D11-E11)</f>
@@ -1640,12 +1646,14 @@
       <c r="B12" s="35" t="n">
         <v>560</v>
       </c>
-      <c r="C12" s="36" t="n"/>
+      <c r="C12" s="36" t="n">
+        <v>407</v>
+      </c>
       <c r="D12" s="23" t="n">
         <v>1350</v>
       </c>
       <c r="E12" s="37" t="n">
-        <v>1712.25</v>
+        <v>1010.92</v>
       </c>
       <c r="F12" s="23">
         <f>IF(E12="","",D12-E12)</f>
@@ -1665,12 +1673,14 @@
       <c r="B13" s="31" t="n">
         <v>650</v>
       </c>
-      <c r="C13" s="32" t="n"/>
+      <c r="C13" s="32" t="n">
+        <v>693</v>
+      </c>
       <c r="D13" s="21" t="n">
         <v>1580</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>1766.51</v>
+        <v>1712.25</v>
       </c>
       <c r="F13" s="21">
         <f>IF(E13="","",D13-E13)</f>
@@ -1690,12 +1700,14 @@
       <c r="B14" s="35" t="n">
         <v>750</v>
       </c>
-      <c r="C14" s="36" t="n"/>
+      <c r="C14" s="36" t="n">
+        <v>751</v>
+      </c>
       <c r="D14" s="23" t="n">
         <v>1800</v>
       </c>
       <c r="E14" s="37" t="n">
-        <v>1804.81</v>
+        <v>1766.51</v>
       </c>
       <c r="F14" s="23">
         <f>IF(E14="","",D14-E14)</f>
@@ -1715,11 +1727,15 @@
       <c r="B15" s="31" t="n">
         <v>850</v>
       </c>
-      <c r="C15" s="32" t="n"/>
+      <c r="C15" s="32" t="n">
+        <v>756</v>
+      </c>
       <c r="D15" s="21" t="n">
         <v>2100</v>
       </c>
-      <c r="E15" s="33" t="n"/>
+      <c r="E15" s="33" t="n">
+        <v>1804.81</v>
+      </c>
       <c r="F15" s="21">
         <f>IF(E15="","",D15-E15)</f>
         <v/>
@@ -1738,7 +1754,9 @@
       <c r="B16" s="35" t="n">
         <v>980</v>
       </c>
-      <c r="C16" s="36" t="n"/>
+      <c r="C16" s="36" t="n">
+        <v>939</v>
+      </c>
       <c r="D16" s="23" t="n">
         <v>2400</v>
       </c>
@@ -1763,11 +1781,15 @@
       <c r="B17" s="31" t="n">
         <v>1120</v>
       </c>
-      <c r="C17" s="32" t="n"/>
+      <c r="C17" s="32" t="n">
+        <v>1002</v>
+      </c>
       <c r="D17" s="21" t="n">
         <v>2750</v>
       </c>
-      <c r="E17" s="33" t="n"/>
+      <c r="E17" s="33" t="n">
+        <v>2312.56</v>
+      </c>
       <c r="F17" s="21">
         <f>IF(E17="","",D17-E17)</f>
         <v/>
@@ -1786,11 +1808,15 @@
       <c r="B18" s="35" t="n">
         <v>1300</v>
       </c>
-      <c r="C18" s="36" t="n"/>
+      <c r="C18" s="36" t="n">
+        <v>1039</v>
+      </c>
       <c r="D18" s="23" t="n">
         <v>3200</v>
       </c>
-      <c r="E18" s="37" t="n"/>
+      <c r="E18" s="37" t="n">
+        <v>2387.26</v>
+      </c>
       <c r="F18" s="23">
         <f>IF(E18="","",D18-E18)</f>
         <v/>
@@ -1809,11 +1835,15 @@
       <c r="B19" s="31" t="n">
         <v>1500</v>
       </c>
-      <c r="C19" s="32" t="n"/>
+      <c r="C19" s="32" t="n">
+        <v>1099</v>
+      </c>
       <c r="D19" s="21" t="n">
         <v>3650</v>
       </c>
-      <c r="E19" s="33" t="n"/>
+      <c r="E19" s="33" t="n">
+        <v>2635.21</v>
+      </c>
       <c r="F19" s="21">
         <f>IF(E19="","",D19-E19)</f>
         <v/>
@@ -4093,13 +4123,13 @@
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>175377</v>
+        <v>166424</v>
       </c>
       <c r="C7" s="21" t="n">
-        <v>175789</v>
+        <v>167269</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>176238</v>
+        <v>168190</v>
       </c>
     </row>
     <row r="8">
@@ -4109,13 +4139,13 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>149641</v>
+        <v>113970</v>
       </c>
       <c r="C8" s="23" t="n">
-        <v>153932</v>
+        <v>122717</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>158126</v>
+        <v>131270</v>
       </c>
     </row>
     <row r="9">
@@ -4125,13 +4155,13 @@
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>106454</v>
+        <v>26295</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>121984</v>
+        <v>57858</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>135580</v>
+        <v>85494</v>
       </c>
     </row>
     <row r="10">
@@ -4141,13 +4171,13 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>41557</v>
+        <v>-105589</v>
       </c>
       <c r="C10" s="23" t="n">
-        <v>80193</v>
+        <v>-27062</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>110478</v>
+        <v>34493</v>
       </c>
     </row>
   </sheetData>

</xml_diff>